<commit_message>
Revised data cleaning and descriptive analysis scripts to focus on All-Stars vs. Non-All-Stars; updated codebook with derived vars; added section at top of report with to-do/items for discussion
</commit_message>
<xml_diff>
--- a/data/nba_codebook.xlsx
+++ b/data/nba_codebook.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emory-my.sharepoint.com/personal/emwu3_emory_edu/Documents/Core/Year 3/DATA 550/Midterm project data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emory-my.sharepoint.com/personal/dtflana_emory_edu/Documents/PhD/Resources/reproducible-research/DATA-550/group_project/data550_midterm/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{8051BF17-FE99-EB4D-933C-48DAD63F5BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF4A853B-C07E-604F-AE6B-AB49564E1D44}"/>
+  <xr:revisionPtr revIDLastSave="193" documentId="8_{8051BF17-FE99-EB4D-933C-48DAD63F5BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6D2F7C3-2050-3E45-BFB3-34EFD01606EE}"/>
   <bookViews>
-    <workbookView xWindow="17940" yWindow="3080" windowWidth="25820" windowHeight="19000" xr2:uid="{FA312644-B801-7B45-9B40-EF4DFDADC3A2}"/>
+    <workbookView xWindow="38400" yWindow="1900" windowWidth="21600" windowHeight="25280" activeTab="1" xr2:uid="{FA312644-B801-7B45-9B40-EF4DFDADC3A2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="old" sheetId="1" r:id="rId1"/>
+    <sheet name="new" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,10 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
-  <si>
-    <t xml:space="preserve"> Rank</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="147">
   <si>
     <t xml:space="preserve"> Position</t>
   </si>
@@ -222,13 +220,271 @@
   </si>
   <si>
     <t>Effective Field Goal Percentage</t>
+  </si>
+  <si>
+    <t>Rank</t>
+  </si>
+  <si>
+    <t>Rk</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>POS</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>GS</t>
+  </si>
+  <si>
+    <t>MP</t>
+  </si>
+  <si>
+    <t>FG</t>
+  </si>
+  <si>
+    <t>FGA</t>
+  </si>
+  <si>
+    <t>FG.</t>
+  </si>
+  <si>
+    <t>X3P</t>
+  </si>
+  <si>
+    <t>X3PA</t>
+  </si>
+  <si>
+    <t>X3P.</t>
+  </si>
+  <si>
+    <t>X2P</t>
+  </si>
+  <si>
+    <t>X2PA</t>
+  </si>
+  <si>
+    <t>X2P.</t>
+  </si>
+  <si>
+    <t>eFG.</t>
+  </si>
+  <si>
+    <t>FT</t>
+  </si>
+  <si>
+    <t>FTA</t>
+  </si>
+  <si>
+    <t>FT.</t>
+  </si>
+  <si>
+    <t>ORB</t>
+  </si>
+  <si>
+    <t>DRB</t>
+  </si>
+  <si>
+    <t>TRB</t>
+  </si>
+  <si>
+    <t>AST</t>
+  </si>
+  <si>
+    <t>STL</t>
+  </si>
+  <si>
+    <t>BLK</t>
+  </si>
+  <si>
+    <t>TOV</t>
+  </si>
+  <si>
+    <t>PF</t>
+  </si>
+  <si>
+    <t>PTS</t>
+  </si>
+  <si>
+    <t>Awards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awards </t>
+  </si>
+  <si>
+    <t>Player's age on February 1 of the season</t>
+  </si>
+  <si>
+    <t>Games</t>
+  </si>
+  <si>
+    <t>Games Started</t>
+  </si>
+  <si>
+    <t>Minutes Played</t>
+  </si>
+  <si>
+    <t>Field Goals Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Field Goal Attempts Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Field Goal Percentage</t>
+  </si>
+  <si>
+    <t>3-Point Field Goal Attempts Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>3-Point Field Goal Percentage</t>
+  </si>
+  <si>
+    <t>2-Point Field Goals Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>2-Point Field Goal Attempts Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>2-Point Field Goal Percentage</t>
+  </si>
+  <si>
+    <t>Free Throws Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Free Throw Attempts Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Free Throw Percentage</t>
+  </si>
+  <si>
+    <t>Offensive Rebounds Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Defensive Rebounds Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Total Rebounds Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Assists Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Steals Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Blocks Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Turnovers Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Personal Fouls Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Points Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>3-Point Field Goals Per 36 Minutes</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>raw_data</t>
+  </si>
+  <si>
+    <t>derived</t>
+  </si>
+  <si>
+    <t>conference</t>
+  </si>
+  <si>
+    <t>Conference</t>
+  </si>
+  <si>
+    <t>division</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>continuous</t>
+  </si>
+  <si>
+    <t>character</t>
+  </si>
+  <si>
+    <t>Values</t>
+  </si>
+  <si>
+    <t>Division</t>
+  </si>
+  <si>
+    <t>categorical</t>
+  </si>
+  <si>
+    <t>1=East, 2=West</t>
+  </si>
+  <si>
+    <t>1=Atlantic, 2=Central, 3=Southeast, 4=Northwest, 5=Pacific, 6=Southwest</t>
+  </si>
+  <si>
+    <t>POS_cat</t>
+  </si>
+  <si>
+    <t>Position (character)</t>
+  </si>
+  <si>
+    <t>Position (categorical)</t>
+  </si>
+  <si>
+    <t>1=PG, 2=SG, 3=SF, 4=PF, 5=C</t>
+  </si>
+  <si>
+    <t>binary</t>
+  </si>
+  <si>
+    <t>All Star (binary)</t>
+  </si>
+  <si>
+    <t>all_star</t>
+  </si>
+  <si>
+    <t>1=Yes, 0=No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS. </t>
+  </si>
+  <si>
+    <t>% Games Started</t>
+  </si>
+  <si>
+    <t>=(GS/G)</t>
+  </si>
+  <si>
+    <t>Var Name (NEW)</t>
+  </si>
+  <si>
+    <t>Rank order is assigned based on number of minutes played (MP)</t>
+  </si>
+  <si>
+    <t>rank_topbottom10</t>
+  </si>
+  <si>
+    <t>Top/Bottom 10 Ranked Players</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -241,6 +497,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -264,14 +527,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -610,253 +896,937 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" t="s">
         <v>60</v>
-      </c>
-      <c r="B19" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CCA1A66-0C69-3D49-B9BD-E8B862546806}">
+  <dimension ref="A1:F38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D9" t="s">
+        <v>120</v>
+      </c>
+      <c r="E9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12" t="s">
+        <v>120</v>
+      </c>
+      <c r="E12" t="s">
+        <v>125</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s">
+        <v>97</v>
+      </c>
+      <c r="D14" t="s">
+        <v>119</v>
+      </c>
+      <c r="E14" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E15" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" t="s">
+        <v>99</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" t="s">
+        <v>119</v>
+      </c>
+      <c r="E17" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" t="s">
+        <v>100</v>
+      </c>
+      <c r="D18" t="s">
+        <v>119</v>
+      </c>
+      <c r="E18" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" t="s">
+        <v>119</v>
+      </c>
+      <c r="E19" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" t="s">
+        <v>102</v>
+      </c>
+      <c r="D20" t="s">
+        <v>119</v>
+      </c>
+      <c r="E20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>78</v>
+      </c>
+      <c r="C23" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" t="s">
+        <v>119</v>
+      </c>
+      <c r="E23" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" t="s">
+        <v>119</v>
+      </c>
+      <c r="E24" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" t="s">
+        <v>119</v>
+      </c>
+      <c r="E25" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" t="s">
+        <v>119</v>
+      </c>
+      <c r="E26" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E27" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" t="s">
+        <v>109</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E28" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D29" t="s">
+        <v>119</v>
+      </c>
+      <c r="E29" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" t="s">
+        <v>111</v>
+      </c>
+      <c r="D30" t="s">
+        <v>119</v>
+      </c>
+      <c r="E30" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>86</v>
+      </c>
+      <c r="C31" t="s">
+        <v>112</v>
+      </c>
+      <c r="D31" t="s">
+        <v>119</v>
+      </c>
+      <c r="E31" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" t="s">
+        <v>113</v>
+      </c>
+      <c r="D32" t="s">
+        <v>119</v>
+      </c>
+      <c r="E32" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E33" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" t="s">
+        <v>115</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E34" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>90</v>
+      </c>
+      <c r="C35" t="s">
+        <v>116</v>
+      </c>
+      <c r="D35" t="s">
+        <v>119</v>
+      </c>
+      <c r="E35" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" t="s">
+        <v>92</v>
+      </c>
+      <c r="D36" t="s">
+        <v>119</v>
+      </c>
+      <c r="E36" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" t="s">
+        <v>137</v>
+      </c>
+      <c r="D37" t="s">
+        <v>120</v>
+      </c>
+      <c r="E37" t="s">
+        <v>136</v>
+      </c>
+      <c r="F37" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>145</v>
+      </c>
+      <c r="C38" t="s">
+        <v>146</v>
+      </c>
+      <c r="D38" t="s">
+        <v>120</v>
+      </c>
+      <c r="E38" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"derived"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>